<commit_message>
feat(productos): Kit de Tareas Hamburguesería v2.0 — 11 ficheros regenerados con el motor de familia 2.4 + contenido propio (canario de los hermanos «▸»): 346 tareas, DV unificada, contador honesto, arqueo con fondo, Trimestral y Anual; idempotencia 0, cache 139/139, censo 0, gate offline 11/11
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/kit-tareas-hamburgueseria/01-apertura-cierre.xlsx
+++ b/astro-site/public/dl/kit-tareas-hamburgueseria/01-apertura-cierre.xlsx
@@ -14,14 +14,15 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cierre Sala" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Instrucciones'!$A$1:$B$33</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Apertura Cocina'!$4:$4</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="1">'Apertura Cocina'!$A$1:$G$36</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Apertura Cocina'!$A$1:$G$50</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Apertura Sala'!$4:$4</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">'Apertura Sala'!$A$1:$G$27</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'Apertura Sala'!$A$1:$G$32</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Cierre Cocina'!$4:$4</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="3">'Cierre Cocina'!$A$1:$G$30</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="3">'Cierre Cocina'!$A$1:$G$37</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Cierre Sala'!$4:$4</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="4">'Cierre Sala'!$A$1:$G$23</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="4">'Cierre Sala'!$A$1:$G$28</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -30,7 +31,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="12">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -92,8 +93,22 @@
       <color rgb="00666666"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFD700"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00333333"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <color rgb="00555555"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -124,6 +139,11 @@
         <bgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8F5E9"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -151,7 +171,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -187,6 +207,49 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <protection locked="0" hidden="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -564,65 +627,166 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="4" customWidth="1" min="1" max="1"/>
-    <col width="80" customWidth="1" min="2" max="2"/>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="100" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1"/>
-    <row r="2">
-      <c r="B2" s="1" t="inlineStr">
+    <row r="2" ht="26" customHeight="1">
+      <c r="B2" s="20" t="inlineStr">
         <is>
           <t>Tareas de Apertura y Cierre — Hamburguesería</t>
         </is>
       </c>
     </row>
     <row r="3"/>
-    <row r="4">
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Checklists diarios para abrir y cerrar cada área de tu hamburguesería.</t>
+    <row r="4" ht="18" customHeight="1">
+      <c r="B4" s="21" t="inlineStr">
+        <is>
+          <t>Cómo cuenta el contador</t>
         </is>
       </c>
     </row>
     <row r="5"/>
-    <row r="6">
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>• Imprime una copia por día y área</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>• Personaliza: borra lo que no aplique, añade lo tuyo</t>
-        </is>
-      </c>
-    </row>
-    <row r="8"/>
+    <row r="6" ht="32" customHeight="1">
+      <c r="B6" s="22" t="inlineStr">
+        <is>
+          <t>▸ Marca con ✓ en la columna «✓ Completada» (desplegable): es la que cuenta el total de tareas completadas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="32" customHeight="1">
+      <c r="B7" s="22" t="inlineStr">
+        <is>
+          <t>▸ «N/A» = no aplica en tu local: esa tarea SALE del total (no la borres, márcala N/A). «—» = no hecha: sigue contando como pendiente y baja el porcentaje, que es de lo que se trata.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="32" customHeight="1">
+      <c r="B8" s="22" t="inlineStr">
+        <is>
+          <t>▸ El denominador cuenta las tareas escritas en la columna «Tarea», no un número fijo: si añades o borras tareas, el total se ajusta solo.</t>
+        </is>
+      </c>
+    </row>
     <row r="9">
-      <c r="B9" s="3" t="inlineStr">
-        <is>
-          <t>Formato: ☐ = pendiente · ✓ = completada</t>
-        </is>
-      </c>
-    </row>
-    <row r="10"/>
+      <c r="B9" s="3" t="n"/>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="B10" s="21" t="inlineStr">
+        <is>
+          <t>Filas libres</t>
+        </is>
+      </c>
+    </row>
     <row r="11">
-      <c r="B11" s="3" t="inlineStr">
-        <is>
-          <t>Marca con ✓ en la columna «✓ Completada» (desplegable): es la que cuenta el total de tareas completadas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12"/>
-    <row r="13">
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>Versión 1.1 · agosto 2026 · aichef.pro/kit-tareas-hamburgueseria · info@aichef.pro</t>
+      <c r="B11" s="3" t="n"/>
+    </row>
+    <row r="12" ht="32" customHeight="1">
+      <c r="B12" s="22" t="inlineStr">
+        <is>
+          <t>▸ Al final de cada tabla hay 5 filas verdes libres DENTRO del rango que cuenta el contador: escribe ahí tus tareas propias.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="32" customHeight="1">
+      <c r="B13" s="22" t="inlineStr">
+        <is>
+          <t>▸ Si necesitas más, inserta filas DENTRO de la tabla (clic derecho → Insertar), nunca por debajo de la última: lo que se escriba fuera del rango no lo cuenta nadie.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="B15" s="21" t="inlineStr">
+        <is>
+          <t>Protección de la hoja</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="32" customHeight="1">
+      <c r="B17" s="22" t="inlineStr">
+        <is>
+          <t>▸ Las hojas con fórmulas van protegidas SIN contraseña: las celdas de entrada (las verdes) están desbloqueadas y los cálculos no se pisan por accidente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="32" customHeight="1">
+      <c r="B18" s="22" t="inlineStr">
+        <is>
+          <t>▸ Puedes insertar y borrar filas con la protección puesta. Para cambiar la estructura: Revisar → Desproteger hoja.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="B20" s="21" t="inlineStr">
+        <is>
+          <t>Se conecta con</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="16" customHeight="1">
+      <c r="B22" s="22" t="inlineStr">
+        <is>
+          <t>▸ 08-apertura-cierre-negocio.xlsx — checklist del LOCAL completo: es el MARCO del día.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="16" customHeight="1">
+      <c r="B23" s="22" t="inlineStr">
+        <is>
+          <t>▸ 01-apertura-cierre.xlsx — el mismo día con el DETALLE por área (cocina, sala).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="16" customHeight="1">
+      <c r="B24" s="22" t="inlineStr">
+        <is>
+          <t>▸ 09-apertura-cierre-caja.xlsx — la CAJA: fondo, recuento por denominaciones, Z del TPV y descuadre.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="48" customHeight="1">
+      <c r="B25" s="22" t="inlineStr">
+        <is>
+          <t>▸ Orden de uso: local → áreas → caja. Cada fichero cubre un nivel: el de negocio marca el HITO (encender, abrir, cerrar), el de áreas detalla CÓMO se hace en cada zona y el de caja lleva el DINERO. Si una tarea aparece en dos, es a propósito: una es el hito y la otra el detalle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="32" customHeight="1">
+      <c r="B26" s="22" t="inlineStr">
+        <is>
+          <t>▸ Estás en 01-apertura-cierre.xlsx: es una capa MÁS, no una repetición — el marco del día está en 08-apertura-cierre-negocio.xlsx.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="18" customHeight="1">
+      <c r="B28" s="21" t="inlineStr">
+        <is>
+          <t>— Kit de Tareas Recurrentes · Hamburguesería · AI Chef Pro · aichef.pro</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="35" customHeight="1">
+      <c r="B30" s="21" t="inlineStr">
+        <is>
+          <t>Diseñado por John Guerrero — chef y consultor gastronómico desde 2010, en cocina desde los 17 años · johnguerrero.es</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="18" customHeight="1">
+      <c r="B31" s="21" t="inlineStr">
+        <is>
+          <t>Contacto: info@aichef.pro</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="18" customHeight="1">
+      <c r="B33" s="21" t="inlineStr">
+        <is>
+          <t>Versión 2.0 · agosto 2026 · aichef.pro/kit-tareas-hamburgueseria · info@aichef.pro</t>
         </is>
       </c>
     </row>
@@ -647,7 +811,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G36"/>
+  <dimension ref="A1:G50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -712,682 +876,983 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  HIGIENE PERSONAL</t>
+        </is>
+      </c>
+      <c r="B5" s="24" t="n"/>
+      <c r="C5" s="24" t="n"/>
+      <c r="D5" s="24" t="n"/>
+      <c r="E5" s="24" t="n"/>
+      <c r="F5" s="24" t="n"/>
+      <c r="G5" s="24" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" s="26" t="inlineStr">
+        <is>
+          <t>Uniforme y calzado de trabajo limpios, delantal cambiado y pelo recogido (gorro o redecilla)</t>
+        </is>
+      </c>
+      <c r="C6" s="27" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D6" s="27" t="inlineStr">
+        <is>
+          <t>Todo el equipo</t>
+        </is>
+      </c>
+      <c r="E6" s="27" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="F6" s="28" t="n"/>
+      <c r="G6" s="28" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="25" t="n">
+        <v>2</v>
+      </c>
+      <c r="B7" s="26" t="inlineStr">
+        <is>
+          <t>Sin anillos, reloj ni pulseras; uñas cortas, limpias y sin esmalte: la carne picada y el montaje se tocan a mano</t>
+        </is>
+      </c>
+      <c r="C7" s="27" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D7" s="27" t="inlineStr">
+        <is>
+          <t>Todo el equipo</t>
+        </is>
+      </c>
+      <c r="E7" s="27" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="F7" s="28" t="n"/>
+      <c r="G7" s="28" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="B8" s="26" t="inlineStr">
+        <is>
+          <t>Heridas y cortes cubiertos con apósito impermeable de color visible y guante encima</t>
+        </is>
+      </c>
+      <c r="C8" s="27" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D8" s="27" t="inlineStr">
+        <is>
+          <t>Todo el equipo</t>
+        </is>
+      </c>
+      <c r="E8" s="27" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="F8" s="28" t="n"/>
+      <c r="G8" s="28" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="25" t="n">
+        <v>4</v>
+      </c>
+      <c r="B9" s="26" t="inlineStr">
+        <is>
+          <t>Lavado de manos al entrar y en cada cambio de tarea; lavamanos con jabón, papel y agua caliente</t>
+        </is>
+      </c>
+      <c r="C9" s="27" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D9" s="27" t="inlineStr">
+        <is>
+          <t>Todo el equipo</t>
+        </is>
+      </c>
+      <c r="E9" s="27" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="F9" s="28" t="n"/>
+      <c r="G9" s="28" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="25" t="n">
+        <v>5</v>
+      </c>
+      <c r="B10" s="26" t="inlineStr">
+        <is>
+          <t>Declarar síntomas digestivos o respiratorios: quien los tenga no manipula alimentos</t>
+        </is>
+      </c>
+      <c r="C10" s="27" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D10" s="27" t="inlineStr">
+        <is>
+          <t>Cocinero</t>
+        </is>
+      </c>
+      <c r="E10" s="27" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="F10" s="28" t="n"/>
+      <c r="G10" s="28" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">  PLANCHA Y FREIDORA</t>
         </is>
       </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="18" t="n">
-        <v>1</v>
-      </c>
-      <c r="B6" s="8" t="inlineStr">
-        <is>
-          <t>Encender plancha/grill y precalentar (200-230°C)</t>
-        </is>
-      </c>
-      <c r="C6" s="9" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D6" s="9" t="inlineStr">
-        <is>
-          <t>Cocinero</t>
-        </is>
-      </c>
-      <c r="E6" s="9" t="inlineStr">
+      <c r="B11" s="24" t="n"/>
+      <c r="C11" s="24" t="n"/>
+      <c r="D11" s="24" t="n"/>
+      <c r="E11" s="24" t="n"/>
+      <c r="F11" s="24" t="n"/>
+      <c r="G11" s="24" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="25" t="n">
+        <v>6</v>
+      </c>
+      <c r="B12" s="26" t="inlineStr">
+        <is>
+          <t>Encender la campana extractora y ventilar la cocina ANTES que ningún equipo: la plancha y la freidora son los dos focos de humo y grasa del local</t>
+        </is>
+      </c>
+      <c r="C12" s="27" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D12" s="27" t="inlineStr">
+        <is>
+          <t>Cocinero</t>
+        </is>
+      </c>
+      <c r="E12" s="27" t="inlineStr">
+        <is>
+          <t>10:45</t>
+        </is>
+      </c>
+      <c r="F12" s="28" t="n"/>
+      <c r="G12" s="28" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="25" t="n">
+        <v>7</v>
+      </c>
+      <c r="B13" s="26" t="inlineStr">
+        <is>
+          <t>Abrir la llave general de gas y comprobar que NO huele a gas antes de prender nada; si huele, no enciendas ni la luz, ventila y avisa al mantenedor</t>
+        </is>
+      </c>
+      <c r="C13" s="27" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D13" s="27" t="inlineStr">
+        <is>
+          <t>Cocinero</t>
+        </is>
+      </c>
+      <c r="E13" s="27" t="inlineStr">
+        <is>
+          <t>10:45</t>
+        </is>
+      </c>
+      <c r="F13" s="28" t="n"/>
+      <c r="G13" s="28" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="25" t="n">
+        <v>8</v>
+      </c>
+      <c r="B14" s="26" t="inlineStr">
+        <is>
+          <t>Encender plancha/grill y precalentar (200-230 °C)</t>
+        </is>
+      </c>
+      <c r="C14" s="27" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D14" s="27" t="inlineStr">
+        <is>
+          <t>Cocinero</t>
+        </is>
+      </c>
+      <c r="E14" s="27" t="inlineStr">
         <is>
           <t>11:00</t>
         </is>
       </c>
-      <c r="F6" s="10" t="n"/>
-      <c r="G6" s="10" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="19" t="n">
-        <v>2</v>
-      </c>
-      <c r="B7" s="12" t="inlineStr">
+      <c r="F14" s="28" t="n"/>
+      <c r="G14" s="28" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="29" t="n">
+        <v>9</v>
+      </c>
+      <c r="B15" s="30" t="inlineStr">
         <is>
           <t>Encender freidora y verificar nivel de aceite</t>
         </is>
       </c>
-      <c r="C7" s="13" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D7" s="13" t="inlineStr">
-        <is>
-          <t>Cocinero</t>
-        </is>
-      </c>
-      <c r="E7" s="13" t="inlineStr">
+      <c r="C15" s="27" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D15" s="27" t="inlineStr">
+        <is>
+          <t>Cocinero</t>
+        </is>
+      </c>
+      <c r="E15" s="27" t="inlineStr">
         <is>
           <t>11:00</t>
         </is>
       </c>
-      <c r="F7" s="14" t="n"/>
-      <c r="G7" s="14" t="n"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="18" t="n">
-        <v>3</v>
-      </c>
-      <c r="B8" s="8" t="inlineStr">
-        <is>
-          <t>Verificar temperatura del aceite (175-180°C para patatas)</t>
-        </is>
-      </c>
-      <c r="C8" s="9" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D8" s="9" t="inlineStr">
-        <is>
-          <t>Cocinero</t>
-        </is>
-      </c>
-      <c r="E8" s="9" t="inlineStr">
+      <c r="F15" s="28" t="n"/>
+      <c r="G15" s="28" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="25" t="n">
+        <v>10</v>
+      </c>
+      <c r="B16" s="26" t="inlineStr">
+        <is>
+          <t>Verificar temperatura del aceite (175-180 °C para patatas)</t>
+        </is>
+      </c>
+      <c r="C16" s="27" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D16" s="27" t="inlineStr">
+        <is>
+          <t>Cocinero</t>
+        </is>
+      </c>
+      <c r="E16" s="27" t="inlineStr">
         <is>
           <t>11:15</t>
         </is>
       </c>
-      <c r="F8" s="10" t="n"/>
-      <c r="G8" s="10" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="19" t="n">
-        <v>4</v>
-      </c>
-      <c r="B9" s="12" t="inlineStr">
-        <is>
-          <t>Encender campana extractora</t>
-        </is>
-      </c>
-      <c r="C9" s="13" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D9" s="13" t="inlineStr">
-        <is>
-          <t>Cocinero</t>
-        </is>
-      </c>
-      <c r="E9" s="13" t="inlineStr">
+      <c r="F16" s="28" t="n"/>
+      <c r="G16" s="28" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="29" t="n">
+        <v>11</v>
+      </c>
+      <c r="B17" s="30" t="inlineStr">
+        <is>
+          <t>Comprobar que la campana tira de verdad (una servilleta pegada a la rejilla se queda sujeta) y que los filtros están puestos y limpios</t>
+        </is>
+      </c>
+      <c r="C17" s="27" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D17" s="27" t="inlineStr">
+        <is>
+          <t>Cocinero</t>
+        </is>
+      </c>
+      <c r="E17" s="27" t="inlineStr">
         <is>
           <t>11:00</t>
         </is>
       </c>
-      <c r="F9" s="14" t="n"/>
-      <c r="G9" s="14" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="18" t="n">
-        <v>5</v>
-      </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="F17" s="28" t="n"/>
+      <c r="G17" s="28" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="25" t="n">
+        <v>12</v>
+      </c>
+      <c r="B18" s="26" t="inlineStr">
         <is>
           <t>Encender horno para panecillos si se tuestan al horno</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D10" s="9" t="inlineStr">
-        <is>
-          <t>Cocinero</t>
-        </is>
-      </c>
-      <c r="E10" s="9" t="inlineStr">
+      <c r="C18" s="27" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D18" s="27" t="inlineStr">
+        <is>
+          <t>Cocinero</t>
+        </is>
+      </c>
+      <c r="E18" s="27" t="inlineStr">
         <is>
           <t>11:00</t>
         </is>
       </c>
-      <c r="F10" s="10" t="n"/>
-      <c r="G10" s="10" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="F18" s="28" t="n"/>
+      <c r="G18" s="28" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">  MISE EN PLACE BURGERS</t>
         </is>
       </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="18" t="n">
-        <v>6</v>
-      </c>
-      <c r="B12" s="8" t="inlineStr">
+      <c r="B19" s="24" t="n"/>
+      <c r="C19" s="24" t="n"/>
+      <c r="D19" s="24" t="n"/>
+      <c r="E19" s="24" t="n"/>
+      <c r="F19" s="24" t="n"/>
+      <c r="G19" s="24" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="25" t="n">
+        <v>13</v>
+      </c>
+      <c r="B20" s="26" t="inlineStr">
+        <is>
+          <t>Comprobar que las cámaras han funcionado toda la noche y registrar temperatura (refrigeración 0-4 °C / congelación ≤ −18 °C) — anota la lectura: ____ °C. Si hay desviación, no uses la carne ni el género hasta valorarlo</t>
+        </is>
+      </c>
+      <c r="C20" s="27" t="inlineStr">
+        <is>
+          <t>Cámara</t>
+        </is>
+      </c>
+      <c r="D20" s="27" t="inlineStr">
+        <is>
+          <t>Cocinero</t>
+        </is>
+      </c>
+      <c r="E20" s="27" t="inlineStr">
+        <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="F20" s="28" t="n"/>
+      <c r="G20" s="28" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="25" t="n">
+        <v>14</v>
+      </c>
+      <c r="B21" s="26" t="inlineStr">
         <is>
           <t>Sacar carne picada/smash patties de cámara (temperar)</t>
         </is>
       </c>
-      <c r="C12" s="9" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D12" s="9" t="inlineStr">
-        <is>
-          <t>Cocinero</t>
-        </is>
-      </c>
-      <c r="E12" s="9" t="inlineStr">
+      <c r="C21" s="27" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D21" s="27" t="inlineStr">
+        <is>
+          <t>Cocinero</t>
+        </is>
+      </c>
+      <c r="E21" s="27" t="inlineStr">
         <is>
           <t>10:30</t>
         </is>
       </c>
-      <c r="F12" s="10" t="n"/>
-      <c r="G12" s="10" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="19" t="n">
-        <v>7</v>
-      </c>
-      <c r="B13" s="12" t="inlineStr">
+      <c r="F21" s="28" t="n"/>
+      <c r="G21" s="28" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="29" t="n">
+        <v>15</v>
+      </c>
+      <c r="B22" s="30" t="inlineStr">
         <is>
           <t>Porcionar carne si se hacen smash burgers al momento</t>
         </is>
       </c>
-      <c r="C13" s="13" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D13" s="13" t="inlineStr">
-        <is>
-          <t>Cocinero</t>
-        </is>
-      </c>
-      <c r="E13" s="13" t="inlineStr">
+      <c r="C22" s="27" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D22" s="27" t="inlineStr">
+        <is>
+          <t>Cocinero</t>
+        </is>
+      </c>
+      <c r="E22" s="27" t="inlineStr">
         <is>
           <t>10:30</t>
         </is>
       </c>
-      <c r="F13" s="14" t="n"/>
-      <c r="G13" s="14" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="18" t="n">
-        <v>8</v>
-      </c>
-      <c r="B14" s="8" t="inlineStr">
+      <c r="F22" s="28" t="n"/>
+      <c r="G22" s="28" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="25" t="n">
+        <v>16</v>
+      </c>
+      <c r="B23" s="26" t="inlineStr">
         <is>
           <t>Cortar pan de burger: brioche, pretzel, clásico</t>
         </is>
       </c>
-      <c r="C14" s="9" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D14" s="9" t="inlineStr">
-        <is>
-          <t>Cocinero</t>
-        </is>
-      </c>
-      <c r="E14" s="9" t="inlineStr">
+      <c r="C23" s="27" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D23" s="27" t="inlineStr">
+        <is>
+          <t>Cocinero</t>
+        </is>
+      </c>
+      <c r="E23" s="27" t="inlineStr">
         <is>
           <t>10:30</t>
         </is>
       </c>
-      <c r="F14" s="10" t="n"/>
-      <c r="G14" s="10" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="19" t="n">
-        <v>9</v>
-      </c>
-      <c r="B15" s="12" t="inlineStr">
+      <c r="F23" s="28" t="n"/>
+      <c r="G23" s="28" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="29" t="n">
+        <v>17</v>
+      </c>
+      <c r="B24" s="30" t="inlineStr">
         <is>
           <t>Preparar toppings: lechuga, tomate, cebolla, pepinillos</t>
         </is>
       </c>
-      <c r="C15" s="13" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D15" s="13" t="inlineStr">
-        <is>
-          <t>Cocinero</t>
-        </is>
-      </c>
-      <c r="E15" s="13" t="inlineStr">
+      <c r="C24" s="27" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D24" s="27" t="inlineStr">
+        <is>
+          <t>Cocinero</t>
+        </is>
+      </c>
+      <c r="E24" s="27" t="inlineStr">
         <is>
           <t>10:30</t>
         </is>
       </c>
-      <c r="F15" s="14" t="n"/>
-      <c r="G15" s="14" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="18" t="n">
-        <v>10</v>
-      </c>
-      <c r="B16" s="8" t="inlineStr">
+      <c r="F24" s="28" t="n"/>
+      <c r="G24" s="28" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="25" t="n">
+        <v>18</v>
+      </c>
+      <c r="B25" s="26" t="inlineStr">
         <is>
           <t>Preparar salsas caseras: burger sauce, BBQ, mostaza miel</t>
         </is>
       </c>
-      <c r="C16" s="9" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D16" s="9" t="inlineStr">
-        <is>
-          <t>Cocinero</t>
-        </is>
-      </c>
-      <c r="E16" s="9" t="inlineStr">
+      <c r="C25" s="27" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D25" s="27" t="inlineStr">
+        <is>
+          <t>Cocinero</t>
+        </is>
+      </c>
+      <c r="E25" s="27" t="inlineStr">
         <is>
           <t>10:30</t>
         </is>
       </c>
-      <c r="F16" s="10" t="n"/>
-      <c r="G16" s="10" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="19" t="n">
-        <v>11</v>
-      </c>
-      <c r="B17" s="12" t="inlineStr">
+      <c r="F25" s="28" t="n"/>
+      <c r="G25" s="28" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="29" t="n">
+        <v>19</v>
+      </c>
+      <c r="B26" s="30" t="inlineStr">
         <is>
           <t>Cortar queso: cheddar, gouda, blue cheese, emmental</t>
         </is>
       </c>
-      <c r="C17" s="13" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D17" s="13" t="inlineStr">
-        <is>
-          <t>Cocinero</t>
-        </is>
-      </c>
-      <c r="E17" s="13" t="inlineStr">
+      <c r="C26" s="27" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D26" s="27" t="inlineStr">
+        <is>
+          <t>Cocinero</t>
+        </is>
+      </c>
+      <c r="E26" s="27" t="inlineStr">
         <is>
           <t>10:30</t>
         </is>
       </c>
-      <c r="F17" s="14" t="n"/>
-      <c r="G17" s="14" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="18" t="n">
-        <v>12</v>
-      </c>
-      <c r="B18" s="8" t="inlineStr">
+      <c r="F26" s="28" t="n"/>
+      <c r="G26" s="28" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="25" t="n">
+        <v>20</v>
+      </c>
+      <c r="B27" s="26" t="inlineStr">
         <is>
           <t>Preparar bacon: pre-cocinado o listo para plancha</t>
         </is>
       </c>
-      <c r="C18" s="9" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D18" s="9" t="inlineStr">
-        <is>
-          <t>Cocinero</t>
-        </is>
-      </c>
-      <c r="E18" s="9" t="inlineStr">
+      <c r="C27" s="27" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D27" s="27" t="inlineStr">
+        <is>
+          <t>Cocinero</t>
+        </is>
+      </c>
+      <c r="E27" s="27" t="inlineStr">
         <is>
           <t>10:45</t>
         </is>
       </c>
-      <c r="F18" s="10" t="n"/>
-      <c r="G18" s="10" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="19" t="n">
-        <v>13</v>
-      </c>
-      <c r="B19" s="12" t="inlineStr">
+      <c r="F27" s="28" t="n"/>
+      <c r="G27" s="28" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="29" t="n">
+        <v>21</v>
+      </c>
+      <c r="B28" s="30" t="inlineStr">
         <is>
           <t>Montar línea de montaje: pan → carne → queso → toppings → salsas</t>
         </is>
       </c>
-      <c r="C19" s="13" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D19" s="13" t="inlineStr">
-        <is>
-          <t>Cocinero</t>
-        </is>
-      </c>
-      <c r="E19" s="13" t="inlineStr">
+      <c r="C28" s="27" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D28" s="27" t="inlineStr">
+        <is>
+          <t>Cocinero</t>
+        </is>
+      </c>
+      <c r="E28" s="27" t="inlineStr">
         <is>
           <t>11:00</t>
         </is>
       </c>
-      <c r="F19" s="14" t="n"/>
-      <c r="G19" s="14" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="6" t="inlineStr">
+      <c r="F28" s="28" t="n"/>
+      <c r="G28" s="28" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">  PATATAS Y SIDES</t>
         </is>
       </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="19" t="n">
-        <v>14</v>
-      </c>
-      <c r="B21" s="12" t="inlineStr">
+      <c r="B29" s="24" t="n"/>
+      <c r="C29" s="24" t="n"/>
+      <c r="D29" s="24" t="n"/>
+      <c r="E29" s="24" t="n"/>
+      <c r="F29" s="24" t="n"/>
+      <c r="G29" s="24" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="29" t="n">
+        <v>22</v>
+      </c>
+      <c r="B30" s="30" t="inlineStr">
         <is>
           <t>Cortar patatas frescas o verificar stock de congeladas</t>
         </is>
       </c>
-      <c r="C21" s="13" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D21" s="13" t="inlineStr">
-        <is>
-          <t>Cocinero</t>
-        </is>
-      </c>
-      <c r="E21" s="13" t="inlineStr">
+      <c r="C30" s="27" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D30" s="27" t="inlineStr">
+        <is>
+          <t>Cocinero</t>
+        </is>
+      </c>
+      <c r="E30" s="27" t="inlineStr">
         <is>
           <t>10:30</t>
         </is>
       </c>
-      <c r="F21" s="14" t="n"/>
-      <c r="G21" s="14" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="18" t="n">
-        <v>15</v>
-      </c>
-      <c r="B22" s="8" t="inlineStr">
+      <c r="F30" s="28" t="n"/>
+      <c r="G30" s="28" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="25" t="n">
+        <v>23</v>
+      </c>
+      <c r="B31" s="26" t="inlineStr">
         <is>
           <t>Preparar aros de cebolla (rebozar)</t>
         </is>
       </c>
-      <c r="C22" s="9" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D22" s="9" t="inlineStr">
-        <is>
-          <t>Cocinero</t>
-        </is>
-      </c>
-      <c r="E22" s="9" t="inlineStr">
+      <c r="C31" s="27" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D31" s="27" t="inlineStr">
+        <is>
+          <t>Cocinero</t>
+        </is>
+      </c>
+      <c r="E31" s="27" t="inlineStr">
         <is>
           <t>10:30</t>
         </is>
       </c>
-      <c r="F22" s="10" t="n"/>
-      <c r="G22" s="10" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="19" t="n">
-        <v>16</v>
-      </c>
-      <c r="B23" s="12" t="inlineStr">
+      <c r="F31" s="28" t="n"/>
+      <c r="G31" s="28" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="29" t="n">
+        <v>24</v>
+      </c>
+      <c r="B32" s="30" t="inlineStr">
         <is>
           <t>Preparar coleslaw del día</t>
         </is>
       </c>
-      <c r="C23" s="13" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D23" s="13" t="inlineStr">
-        <is>
-          <t>Cocinero</t>
-        </is>
-      </c>
-      <c r="E23" s="13" t="inlineStr">
+      <c r="C32" s="27" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D32" s="27" t="inlineStr">
+        <is>
+          <t>Cocinero</t>
+        </is>
+      </c>
+      <c r="E32" s="27" t="inlineStr">
         <is>
           <t>10:30</t>
         </is>
       </c>
-      <c r="F23" s="14" t="n"/>
-      <c r="G23" s="14" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="18" t="n">
-        <v>17</v>
-      </c>
-      <c r="B24" s="8" t="inlineStr">
+      <c r="F32" s="28" t="n"/>
+      <c r="G32" s="28" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="25" t="n">
+        <v>25</v>
+      </c>
+      <c r="B33" s="26" t="inlineStr">
         <is>
           <t>Verificar stock de nachos, jalapeños, guacamole</t>
         </is>
       </c>
-      <c r="C24" s="9" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D24" s="9" t="inlineStr">
-        <is>
-          <t>Cocinero</t>
-        </is>
-      </c>
-      <c r="E24" s="9" t="inlineStr">
+      <c r="C33" s="27" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D33" s="27" t="inlineStr">
+        <is>
+          <t>Cocinero</t>
+        </is>
+      </c>
+      <c r="E33" s="27" t="inlineStr">
         <is>
           <t>10:30</t>
         </is>
       </c>
-      <c r="F24" s="10" t="n"/>
-      <c r="G24" s="10" t="n"/>
-    </row>
-    <row r="25">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  STOCK E HIGIENE</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="18" t="n">
-        <v>18</v>
-      </c>
-      <c r="B26" s="8" t="inlineStr">
+      <c r="F33" s="28" t="n"/>
+      <c r="G33" s="28" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  STOCK Y DESINFECCIÓN</t>
+        </is>
+      </c>
+      <c r="B34" s="24" t="n"/>
+      <c r="C34" s="24" t="n"/>
+      <c r="D34" s="24" t="n"/>
+      <c r="E34" s="24" t="n"/>
+      <c r="F34" s="24" t="n"/>
+      <c r="G34" s="24" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="25" t="n">
+        <v>26</v>
+      </c>
+      <c r="B35" s="26" t="inlineStr">
         <is>
           <t>Verificar stock de carne (piezas para el día)</t>
         </is>
       </c>
-      <c r="C26" s="9" t="inlineStr">
+      <c r="C35" s="27" t="inlineStr">
         <is>
           <t>Cámara</t>
         </is>
       </c>
-      <c r="D26" s="9" t="inlineStr">
-        <is>
-          <t>Cocinero</t>
-        </is>
-      </c>
-      <c r="E26" s="9" t="inlineStr">
+      <c r="D35" s="27" t="inlineStr">
+        <is>
+          <t>Cocinero</t>
+        </is>
+      </c>
+      <c r="E35" s="27" t="inlineStr">
         <is>
           <t>10:00</t>
         </is>
       </c>
-      <c r="F26" s="10" t="n"/>
-      <c r="G26" s="10" t="n"/>
-    </row>
-    <row r="27">
-      <c r="A27" s="19" t="n">
-        <v>19</v>
-      </c>
-      <c r="B27" s="12" t="inlineStr">
+      <c r="F35" s="28" t="n"/>
+      <c r="G35" s="28" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="29" t="n">
+        <v>27</v>
+      </c>
+      <c r="B36" s="30" t="inlineStr">
         <is>
           <t>Verificar stock de pan de burger</t>
         </is>
       </c>
-      <c r="C27" s="13" t="inlineStr">
+      <c r="C36" s="27" t="inlineStr">
         <is>
           <t>Almacén</t>
         </is>
       </c>
-      <c r="D27" s="13" t="inlineStr">
-        <is>
-          <t>Cocinero</t>
-        </is>
-      </c>
-      <c r="E27" s="13" t="inlineStr">
+      <c r="D36" s="27" t="inlineStr">
+        <is>
+          <t>Cocinero</t>
+        </is>
+      </c>
+      <c r="E36" s="27" t="inlineStr">
         <is>
           <t>10:00</t>
         </is>
       </c>
-      <c r="F27" s="14" t="n"/>
-      <c r="G27" s="14" t="n"/>
-    </row>
-    <row r="28">
-      <c r="A28" s="18" t="n">
-        <v>20</v>
-      </c>
-      <c r="B28" s="8" t="inlineStr">
+      <c r="F36" s="28" t="n"/>
+      <c r="G36" s="28" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="25" t="n">
+        <v>28</v>
+      </c>
+      <c r="B37" s="26" t="inlineStr">
         <is>
           <t>Verificar caducidades de productos abiertos</t>
         </is>
       </c>
-      <c r="C28" s="9" t="inlineStr">
+      <c r="C37" s="27" t="inlineStr">
         <is>
           <t>Cámara</t>
         </is>
       </c>
-      <c r="D28" s="9" t="inlineStr">
-        <is>
-          <t>Cocinero</t>
-        </is>
-      </c>
-      <c r="E28" s="9" t="inlineStr">
+      <c r="D37" s="27" t="inlineStr">
+        <is>
+          <t>Cocinero</t>
+        </is>
+      </c>
+      <c r="E37" s="27" t="inlineStr">
         <is>
           <t>10:00</t>
         </is>
       </c>
-      <c r="F28" s="10" t="n"/>
-      <c r="G28" s="10" t="n"/>
-    </row>
-    <row r="29">
-      <c r="A29" s="19" t="n">
-        <v>21</v>
-      </c>
-      <c r="B29" s="12" t="inlineStr">
-        <is>
-          <t>Lavarse manos, uniforme completo</t>
-        </is>
-      </c>
-      <c r="C29" s="13" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D29" s="13" t="inlineStr">
+      <c r="F37" s="28" t="n"/>
+      <c r="G37" s="28" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="29" t="n">
+        <v>29</v>
+      </c>
+      <c r="B38" s="30" t="inlineStr">
+        <is>
+          <t>Lavarse las manos y cambiar de guantes al pasar de la carne CRUDA al pan, los toppings o las salsas; tabla, pinzas y espátula de crudo no vuelven a la línea de montaje</t>
+        </is>
+      </c>
+      <c r="C38" s="27" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D38" s="27" t="inlineStr">
         <is>
           <t>Todos</t>
         </is>
       </c>
-      <c r="E29" s="13" t="inlineStr">
+      <c r="E38" s="27" t="inlineStr">
         <is>
           <t>10:00</t>
         </is>
       </c>
-      <c r="F29" s="14" t="n"/>
-      <c r="G29" s="14" t="n"/>
-    </row>
-    <row r="30">
-      <c r="A30" s="18" t="n">
-        <v>22</v>
-      </c>
-      <c r="B30" s="8" t="inlineStr">
+      <c r="F38" s="28" t="n"/>
+      <c r="G38" s="28" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="25" t="n">
+        <v>30</v>
+      </c>
+      <c r="B39" s="26" t="inlineStr">
         <is>
           <t>Desinfectar superficies de trabajo</t>
         </is>
       </c>
-      <c r="C30" s="9" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D30" s="9" t="inlineStr">
-        <is>
-          <t>Cocinero</t>
-        </is>
-      </c>
-      <c r="E30" s="9" t="inlineStr">
+      <c r="C39" s="27" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D39" s="27" t="inlineStr">
+        <is>
+          <t>Cocinero</t>
+        </is>
+      </c>
+      <c r="E39" s="27" t="inlineStr">
         <is>
           <t>10:00</t>
         </is>
       </c>
-      <c r="F30" s="10" t="n"/>
-      <c r="G30" s="10" t="n"/>
-    </row>
-    <row r="31"/>
-    <row r="32">
-      <c r="C32" s="15" t="inlineStr">
-        <is>
-          <t>Completadas:</t>
-        </is>
-      </c>
-      <c r="D32" s="16">
-        <f>COUNTIF(F5:F30,"✓")</f>
+      <c r="F39" s="28" t="n"/>
+      <c r="G39" s="28" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="31" t="n"/>
+      <c r="B40" s="32" t="n"/>
+      <c r="C40" s="27" t="n"/>
+      <c r="D40" s="27" t="n"/>
+      <c r="E40" s="27" t="n"/>
+      <c r="F40" s="28" t="n"/>
+      <c r="G40" s="28" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="31" t="n"/>
+      <c r="B41" s="32" t="n"/>
+      <c r="C41" s="27" t="n"/>
+      <c r="D41" s="27" t="n"/>
+      <c r="E41" s="27" t="n"/>
+      <c r="F41" s="28" t="n"/>
+      <c r="G41" s="28" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="31" t="n"/>
+      <c r="B42" s="32" t="n"/>
+      <c r="C42" s="27" t="n"/>
+      <c r="D42" s="27" t="n"/>
+      <c r="E42" s="27" t="n"/>
+      <c r="F42" s="28" t="n"/>
+      <c r="G42" s="28" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="31" t="n"/>
+      <c r="B43" s="32" t="n"/>
+      <c r="C43" s="27" t="n"/>
+      <c r="D43" s="27" t="n"/>
+      <c r="E43" s="27" t="n"/>
+      <c r="F43" s="28" t="n"/>
+      <c r="G43" s="28" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="31" t="n"/>
+      <c r="B44" s="32" t="n"/>
+      <c r="C44" s="27" t="n"/>
+      <c r="D44" s="27" t="n"/>
+      <c r="E44" s="27" t="n"/>
+      <c r="F44" s="28" t="n"/>
+      <c r="G44" s="28" t="n"/>
+    </row>
+    <row r="45"/>
+    <row r="46">
+      <c r="A46" s="15" t="inlineStr">
+        <is>
+          <t>Tareas completadas:</t>
+        </is>
+      </c>
+      <c r="D46" s="16">
+        <f>COUNTIFS(B5:B44,"?*",F5:F44,"✓")</f>
         <v>0.0</v>
       </c>
-      <c r="E32" s="15" t="inlineStr">
+      <c r="E46" s="15" t="inlineStr">
         <is>
           <t>de</t>
         </is>
       </c>
-      <c r="F32">
-        <f>COUNTIF(B5:B30,"?*")</f>
-        <v>22.0</v>
-      </c>
-    </row>
-    <row r="33"/>
-    <row r="34">
-      <c r="A34" s="4" t="inlineStr">
+      <c r="F46">
+        <f>COUNTIF(B5:B44,"?*")-COUNTIF(F5:F44,"N/A")</f>
+        <v>30.0</v>
+      </c>
+    </row>
+    <row r="47"/>
+    <row r="48">
+      <c r="A48" s="4" t="inlineStr">
         <is>
           <t>Firma encargado/a: _________________________    Hora: _________</t>
         </is>
       </c>
     </row>
-    <row r="35"/>
-    <row r="36">
-      <c r="A36" s="17" t="inlineStr">
-        <is>
-          <t>— Kit de Tareas Recurrentes: Hamburguesería · AI Chef Pro · aichef.pro —</t>
+    <row r="49"/>
+    <row r="50">
+      <c r="A50" s="17" t="inlineStr">
+        <is>
+          <t>— Kit de Tareas Recurrentes · Hamburguesería · AI Chef Pro · aichef.pro</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="A20:G20"/>
-    <mergeCell ref="A36:G36"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="0" formatRows="0" sort="0"/>
+  <mergeCells count="10">
     <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A48:G48"/>
+    <mergeCell ref="A46:C46"/>
+    <mergeCell ref="A19:G19"/>
+    <mergeCell ref="A29:G29"/>
+    <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A50:G50"/>
+    <mergeCell ref="A34:G34"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A34:G34"/>
-    <mergeCell ref="A25:G25"/>
-    <mergeCell ref="A5:G5"/>
     <mergeCell ref="A11:G11"/>
   </mergeCells>
-  <conditionalFormatting sqref="A5:G30">
+  <conditionalFormatting sqref="A5:G44">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$F5="✓"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F6 F7 F8 F9 F10 F12 F13 F14 F15 F16 F17 F18 F19 F21 F22 F23 F24 F26 F27 F28 F29 F30" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F6 F7 F8 F9 F10 F12 F13 F14 F15 F16 F17 F18 F20 F21 F22 F23 F24 F25 F26 F27 F28 F30 F31 F32 F33 F35 F36 F37 F38 F39 F40 F41 F42 F43 F44" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Marca no válida" error="Usa el desplegable: ✓, — o N/A. N/A = no aplica, sale del total; — = no hecha, cuenta como pendiente." type="list" errorStyle="stop">
       <formula1>"✓,—,N/A"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1411,7 +1876,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1476,458 +1941,523 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">  SALA</t>
         </is>
       </c>
+      <c r="B5" s="24" t="n"/>
+      <c r="C5" s="24" t="n"/>
+      <c r="D5" s="24" t="n"/>
+      <c r="E5" s="24" t="n"/>
+      <c r="F5" s="24" t="n"/>
+      <c r="G5" s="24" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="18" t="n">
+      <c r="A6" s="25" t="n">
         <v>1</v>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B6" s="26" t="inlineStr">
         <is>
           <t>Encender luces y climatización</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="C6" s="27" t="inlineStr">
         <is>
           <t>Sala</t>
         </is>
       </c>
-      <c r="D6" s="9" t="inlineStr">
+      <c r="D6" s="27" t="inlineStr">
         <is>
           <t>Camarero/a</t>
         </is>
       </c>
-      <c r="E6" s="9" t="inlineStr">
+      <c r="E6" s="27" t="inlineStr">
         <is>
           <t>11:00</t>
         </is>
       </c>
-      <c r="F6" s="10" t="n"/>
-      <c r="G6" s="10" t="n"/>
+      <c r="F6" s="28" t="n"/>
+      <c r="G6" s="28" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="19" t="n">
+      <c r="A7" s="29" t="n">
         <v>2</v>
       </c>
-      <c r="B7" s="12" t="inlineStr">
+      <c r="B7" s="30" t="inlineStr">
         <is>
           <t>Limpiar y montar mesas</t>
         </is>
       </c>
-      <c r="C7" s="13" t="inlineStr">
+      <c r="C7" s="27" t="inlineStr">
         <is>
           <t>Sala</t>
         </is>
       </c>
-      <c r="D7" s="13" t="inlineStr">
+      <c r="D7" s="27" t="inlineStr">
         <is>
           <t>Camarero/a</t>
         </is>
       </c>
-      <c r="E7" s="13" t="inlineStr">
+      <c r="E7" s="27" t="inlineStr">
         <is>
           <t>11:00</t>
         </is>
       </c>
-      <c r="F7" s="14" t="n"/>
-      <c r="G7" s="14" t="n"/>
+      <c r="F7" s="28" t="n"/>
+      <c r="G7" s="28" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="18" t="n">
+      <c r="A8" s="25" t="n">
         <v>3</v>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B8" s="26" t="inlineStr">
         <is>
           <t>Colocar menús/cartas en mesas y barra</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="C8" s="27" t="inlineStr">
         <is>
           <t>Sala</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr">
+      <c r="D8" s="27" t="inlineStr">
         <is>
           <t>Camarero/a</t>
         </is>
       </c>
-      <c r="E8" s="9" t="inlineStr">
+      <c r="E8" s="27" t="inlineStr">
         <is>
           <t>11:00</t>
         </is>
       </c>
-      <c r="F8" s="10" t="n"/>
-      <c r="G8" s="10" t="n"/>
+      <c r="F8" s="28" t="n"/>
+      <c r="G8" s="28" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="19" t="n">
+      <c r="A9" s="29" t="n">
         <v>4</v>
       </c>
-      <c r="B9" s="12" t="inlineStr">
+      <c r="B9" s="30" t="inlineStr">
         <is>
           <t>Actualizar pizarra: burger del día, combos</t>
         </is>
       </c>
-      <c r="C9" s="13" t="inlineStr">
+      <c r="C9" s="27" t="inlineStr">
         <is>
           <t>Sala</t>
         </is>
       </c>
-      <c r="D9" s="13" t="inlineStr">
+      <c r="D9" s="27" t="inlineStr">
         <is>
           <t>Encargado/a</t>
         </is>
       </c>
-      <c r="E9" s="13" t="inlineStr">
+      <c r="E9" s="27" t="inlineStr">
         <is>
           <t>11:15</t>
         </is>
       </c>
-      <c r="F9" s="14" t="n"/>
-      <c r="G9" s="14" t="n"/>
+      <c r="F9" s="28" t="n"/>
+      <c r="G9" s="28" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="18" t="n">
+      <c r="A10" s="25" t="n">
         <v>5</v>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B10" s="26" t="inlineStr">
         <is>
           <t>Poner música ambiental</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
+      <c r="C10" s="27" t="inlineStr">
         <is>
           <t>Sala</t>
         </is>
       </c>
-      <c r="D10" s="9" t="inlineStr">
+      <c r="D10" s="27" t="inlineStr">
         <is>
           <t>Encargado/a</t>
         </is>
       </c>
-      <c r="E10" s="9" t="inlineStr">
+      <c r="E10" s="27" t="inlineStr">
         <is>
           <t>11:15</t>
         </is>
       </c>
-      <c r="F10" s="10" t="n"/>
-      <c r="G10" s="10" t="n"/>
+      <c r="F10" s="28" t="n"/>
+      <c r="G10" s="28" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="19" t="n">
+      <c r="A11" s="29" t="n">
         <v>6</v>
       </c>
-      <c r="B11" s="12" t="inlineStr">
+      <c r="B11" s="30" t="inlineStr">
         <is>
           <t>Verificar TPV/datáfono</t>
         </is>
       </c>
-      <c r="C11" s="13" t="inlineStr">
+      <c r="C11" s="27" t="inlineStr">
         <is>
           <t>Sala</t>
         </is>
       </c>
-      <c r="D11" s="13" t="inlineStr">
+      <c r="D11" s="27" t="inlineStr">
         <is>
           <t>Encargado/a</t>
         </is>
       </c>
-      <c r="E11" s="13" t="inlineStr">
+      <c r="E11" s="27" t="inlineStr">
         <is>
           <t>11:15</t>
         </is>
       </c>
-      <c r="F11" s="14" t="n"/>
-      <c r="G11" s="14" t="n"/>
+      <c r="F11" s="28" t="n"/>
+      <c r="G11" s="28" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="18" t="n">
+      <c r="A12" s="25" t="n">
         <v>7</v>
       </c>
-      <c r="B12" s="8" t="inlineStr">
+      <c r="B12" s="26" t="inlineStr">
         <is>
           <t>Preparar fondo de caja</t>
         </is>
       </c>
-      <c r="C12" s="9" t="inlineStr">
+      <c r="C12" s="27" t="inlineStr">
         <is>
           <t>Sala</t>
         </is>
       </c>
-      <c r="D12" s="9" t="inlineStr">
+      <c r="D12" s="27" t="inlineStr">
         <is>
           <t>Encargado/a</t>
         </is>
       </c>
-      <c r="E12" s="9" t="inlineStr">
+      <c r="E12" s="27" t="inlineStr">
         <is>
           <t>11:15</t>
         </is>
       </c>
-      <c r="F12" s="10" t="n"/>
-      <c r="G12" s="10" t="n"/>
+      <c r="F12" s="28" t="n"/>
+      <c r="G12" s="28" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="6" t="inlineStr">
+      <c r="A13" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">  DELIVERY Y TAKE-AWAY</t>
         </is>
       </c>
+      <c r="B13" s="24" t="n"/>
+      <c r="C13" s="24" t="n"/>
+      <c r="D13" s="24" t="n"/>
+      <c r="E13" s="24" t="n"/>
+      <c r="F13" s="24" t="n"/>
+      <c r="G13" s="24" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="18" t="n">
+      <c r="A14" s="25" t="n">
         <v>8</v>
       </c>
-      <c r="B14" s="8" t="inlineStr">
+      <c r="B14" s="26" t="inlineStr">
         <is>
           <t>Encender tablets de delivery (Glovo, Uber Eats, Just Eat)</t>
         </is>
       </c>
-      <c r="C14" s="9" t="inlineStr">
+      <c r="C14" s="27" t="inlineStr">
         <is>
           <t>Sala</t>
         </is>
       </c>
-      <c r="D14" s="9" t="inlineStr">
+      <c r="D14" s="27" t="inlineStr">
         <is>
           <t>Encargado/a</t>
         </is>
       </c>
-      <c r="E14" s="9" t="inlineStr">
+      <c r="E14" s="27" t="inlineStr">
         <is>
           <t>11:30</t>
         </is>
       </c>
-      <c r="F14" s="10" t="n"/>
-      <c r="G14" s="10" t="n"/>
+      <c r="F14" s="28" t="n"/>
+      <c r="G14" s="28" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="19" t="n">
+      <c r="A15" s="29" t="n">
         <v>9</v>
       </c>
-      <c r="B15" s="12" t="inlineStr">
+      <c r="B15" s="30" t="inlineStr">
         <is>
           <t>Verificar stock de cajas burger, bolsas, servilletas</t>
         </is>
       </c>
-      <c r="C15" s="13" t="inlineStr">
+      <c r="C15" s="27" t="inlineStr">
         <is>
           <t>Almacén</t>
         </is>
       </c>
-      <c r="D15" s="13" t="inlineStr">
+      <c r="D15" s="27" t="inlineStr">
         <is>
           <t>Encargado/a</t>
         </is>
       </c>
-      <c r="E15" s="13" t="inlineStr">
+      <c r="E15" s="27" t="inlineStr">
         <is>
           <t>11:00</t>
         </is>
       </c>
-      <c r="F15" s="14" t="n"/>
-      <c r="G15" s="14" t="n"/>
+      <c r="F15" s="28" t="n"/>
+      <c r="G15" s="28" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="18" t="n">
+      <c r="A16" s="25" t="n">
         <v>10</v>
       </c>
-      <c r="B16" s="8" t="inlineStr">
+      <c r="B16" s="26" t="inlineStr">
         <is>
           <t>Verificar stock de envases para patatas y sides</t>
         </is>
       </c>
-      <c r="C16" s="9" t="inlineStr">
+      <c r="C16" s="27" t="inlineStr">
         <is>
           <t>Almacén</t>
         </is>
       </c>
-      <c r="D16" s="9" t="inlineStr">
+      <c r="D16" s="27" t="inlineStr">
         <is>
           <t>Encargado/a</t>
         </is>
       </c>
-      <c r="E16" s="9" t="inlineStr">
+      <c r="E16" s="27" t="inlineStr">
         <is>
           <t>11:00</t>
         </is>
       </c>
-      <c r="F16" s="10" t="n"/>
-      <c r="G16" s="10" t="n"/>
+      <c r="F16" s="28" t="n"/>
+      <c r="G16" s="28" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="19" t="n">
+      <c r="A17" s="29" t="n">
         <v>11</v>
       </c>
-      <c r="B17" s="12" t="inlineStr">
+      <c r="B17" s="30" t="inlineStr">
         <is>
           <t>Actualizar menú en apps si hay cambios/86s</t>
         </is>
       </c>
-      <c r="C17" s="13" t="inlineStr">
+      <c r="C17" s="27" t="inlineStr">
         <is>
           <t>Office</t>
         </is>
       </c>
-      <c r="D17" s="13" t="inlineStr">
+      <c r="D17" s="27" t="inlineStr">
         <is>
           <t>Encargado/a</t>
         </is>
       </c>
-      <c r="E17" s="13" t="inlineStr">
+      <c r="E17" s="27" t="inlineStr">
         <is>
           <t>11:00</t>
         </is>
       </c>
-      <c r="F17" s="14" t="n"/>
-      <c r="G17" s="14" t="n"/>
+      <c r="F17" s="28" t="n"/>
+      <c r="G17" s="28" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="6" t="inlineStr">
+      <c r="A18" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">  BAÑOS Y LIMPIEZA</t>
         </is>
       </c>
+      <c r="B18" s="24" t="n"/>
+      <c r="C18" s="24" t="n"/>
+      <c r="D18" s="24" t="n"/>
+      <c r="E18" s="24" t="n"/>
+      <c r="F18" s="24" t="n"/>
+      <c r="G18" s="24" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="19" t="n">
+      <c r="A19" s="29" t="n">
         <v>12</v>
       </c>
-      <c r="B19" s="12" t="inlineStr">
+      <c r="B19" s="30" t="inlineStr">
         <is>
           <t>Barrer y fregar suelo de sala</t>
         </is>
       </c>
-      <c r="C19" s="13" t="inlineStr">
+      <c r="C19" s="27" t="inlineStr">
         <is>
           <t>Sala</t>
         </is>
       </c>
-      <c r="D19" s="13" t="inlineStr">
+      <c r="D19" s="27" t="inlineStr">
         <is>
           <t>Auxiliar</t>
         </is>
       </c>
-      <c r="E19" s="13" t="inlineStr">
+      <c r="E19" s="27" t="inlineStr">
         <is>
           <t>10:30</t>
         </is>
       </c>
-      <c r="F19" s="14" t="n"/>
-      <c r="G19" s="14" t="n"/>
+      <c r="F19" s="28" t="n"/>
+      <c r="G19" s="28" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="18" t="n">
+      <c r="A20" s="25" t="n">
         <v>13</v>
       </c>
-      <c r="B20" s="8" t="inlineStr">
+      <c r="B20" s="26" t="inlineStr">
         <is>
           <t>Limpiar baños: jabón, papel, suelo</t>
         </is>
       </c>
-      <c r="C20" s="9" t="inlineStr">
+      <c r="C20" s="27" t="inlineStr">
         <is>
           <t>Baños</t>
         </is>
       </c>
-      <c r="D20" s="9" t="inlineStr">
+      <c r="D20" s="27" t="inlineStr">
         <is>
           <t>Auxiliar</t>
         </is>
       </c>
-      <c r="E20" s="9" t="inlineStr">
+      <c r="E20" s="27" t="inlineStr">
         <is>
           <t>10:30</t>
         </is>
       </c>
-      <c r="F20" s="10" t="n"/>
-      <c r="G20" s="10" t="n"/>
+      <c r="F20" s="28" t="n"/>
+      <c r="G20" s="28" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="19" t="n">
+      <c r="A21" s="29" t="n">
         <v>14</v>
       </c>
-      <c r="B21" s="12" t="inlineStr">
+      <c r="B21" s="30" t="inlineStr">
         <is>
           <t>Limpiar cristales entrada</t>
         </is>
       </c>
-      <c r="C21" s="13" t="inlineStr">
+      <c r="C21" s="27" t="inlineStr">
         <is>
           <t>Sala</t>
         </is>
       </c>
-      <c r="D21" s="13" t="inlineStr">
+      <c r="D21" s="27" t="inlineStr">
         <is>
           <t>Auxiliar</t>
         </is>
       </c>
-      <c r="E21" s="13" t="inlineStr">
+      <c r="E21" s="27" t="inlineStr">
         <is>
           <t>10:30</t>
         </is>
       </c>
-      <c r="F21" s="14" t="n"/>
-      <c r="G21" s="14" t="n"/>
-    </row>
-    <row r="22"/>
+      <c r="F21" s="28" t="n"/>
+      <c r="G21" s="28" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="31" t="n"/>
+      <c r="B22" s="32" t="n"/>
+      <c r="C22" s="27" t="n"/>
+      <c r="D22" s="27" t="n"/>
+      <c r="E22" s="27" t="n"/>
+      <c r="F22" s="28" t="n"/>
+      <c r="G22" s="28" t="n"/>
+    </row>
     <row r="23">
-      <c r="C23" s="15" t="inlineStr">
-        <is>
-          <t>Completadas:</t>
-        </is>
-      </c>
-      <c r="D23" s="16">
-        <f>COUNTIF(F5:F21,"✓")</f>
+      <c r="A23" s="31" t="n"/>
+      <c r="B23" s="32" t="n"/>
+      <c r="C23" s="27" t="n"/>
+      <c r="D23" s="27" t="n"/>
+      <c r="E23" s="27" t="n"/>
+      <c r="F23" s="28" t="n"/>
+      <c r="G23" s="28" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="31" t="n"/>
+      <c r="B24" s="32" t="n"/>
+      <c r="C24" s="27" t="n"/>
+      <c r="D24" s="27" t="n"/>
+      <c r="E24" s="27" t="n"/>
+      <c r="F24" s="28" t="n"/>
+      <c r="G24" s="28" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="31" t="n"/>
+      <c r="B25" s="32" t="n"/>
+      <c r="C25" s="27" t="n"/>
+      <c r="D25" s="27" t="n"/>
+      <c r="E25" s="27" t="n"/>
+      <c r="F25" s="28" t="n"/>
+      <c r="G25" s="28" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="31" t="n"/>
+      <c r="B26" s="32" t="n"/>
+      <c r="C26" s="27" t="n"/>
+      <c r="D26" s="27" t="n"/>
+      <c r="E26" s="27" t="n"/>
+      <c r="F26" s="28" t="n"/>
+      <c r="G26" s="28" t="n"/>
+    </row>
+    <row r="27"/>
+    <row r="28">
+      <c r="A28" s="15" t="inlineStr">
+        <is>
+          <t>Tareas completadas:</t>
+        </is>
+      </c>
+      <c r="D28" s="16">
+        <f>COUNTIFS(B5:B26,"?*",F5:F26,"✓")</f>
         <v>0.0</v>
       </c>
-      <c r="E23" s="15" t="inlineStr">
+      <c r="E28" s="15" t="inlineStr">
         <is>
           <t>de</t>
         </is>
       </c>
-      <c r="F23">
-        <f>COUNTIF(B5:B21,"?*")</f>
+      <c r="F28">
+        <f>COUNTIF(B5:B26,"?*")-COUNTIF(F5:F26,"N/A")</f>
         <v>14.0</v>
       </c>
     </row>
-    <row r="24"/>
-    <row r="25">
-      <c r="A25" s="4" t="inlineStr">
+    <row r="29"/>
+    <row r="30">
+      <c r="A30" s="4" t="inlineStr">
         <is>
           <t>Firma encargado/a: _________________________    Hora: _________</t>
         </is>
       </c>
     </row>
-    <row r="26"/>
-    <row r="27">
-      <c r="A27" s="17" t="inlineStr">
-        <is>
-          <t>— Kit de Tareas Recurrentes: Hamburguesería · AI Chef Pro · aichef.pro —</t>
+    <row r="31"/>
+    <row r="32">
+      <c r="A32" s="17" t="inlineStr">
+        <is>
+          <t>— Kit de Tareas Recurrentes · Hamburguesería · AI Chef Pro · aichef.pro</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="0" formatRows="0" sort="0"/>
+  <mergeCells count="8">
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A27:G27"/>
+    <mergeCell ref="A32:G32"/>
+    <mergeCell ref="A18:G18"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A18:G18"/>
-    <mergeCell ref="A25:G25"/>
+    <mergeCell ref="A30:G30"/>
     <mergeCell ref="A5:G5"/>
     <mergeCell ref="A13:G13"/>
+    <mergeCell ref="A28:C28"/>
   </mergeCells>
-  <conditionalFormatting sqref="A5:G21">
+  <conditionalFormatting sqref="A5:G26">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$F5="✓"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F6 F7 F8 F9 F10 F11 F12 F14 F15 F16 F17 F19 F20 F21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F6 F7 F8 F9 F10 F11 F12 F14 F15 F16 F17 F19 F20 F21 F22 F23 F24 F25 F26" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Marca no válida" error="Usa el desplegable: ✓, — o N/A. N/A = no aplica, sale del total; — = no hecha, cuenta como pendiente." type="list" errorStyle="stop">
       <formula1>"✓,—,N/A"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1951,7 +2481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2016,520 +2546,645 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">  PRODUCTO</t>
         </is>
       </c>
+      <c r="B5" s="24" t="n"/>
+      <c r="C5" s="24" t="n"/>
+      <c r="D5" s="24" t="n"/>
+      <c r="E5" s="24" t="n"/>
+      <c r="F5" s="24" t="n"/>
+      <c r="G5" s="24" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="18" t="n">
+      <c r="A6" s="25" t="n">
         <v>1</v>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B6" s="26" t="inlineStr">
         <is>
           <t>Guardar carne sobrante en cámara (etiquetar fecha)</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D6" s="9" t="inlineStr">
-        <is>
-          <t>Cocinero</t>
-        </is>
-      </c>
-      <c r="E6" s="9" t="inlineStr">
+      <c r="C6" s="27" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D6" s="27" t="inlineStr">
+        <is>
+          <t>Cocinero</t>
+        </is>
+      </c>
+      <c r="E6" s="27" t="inlineStr">
         <is>
           <t>22:30</t>
         </is>
       </c>
-      <c r="F6" s="10" t="n"/>
-      <c r="G6" s="10" t="n"/>
+      <c r="F6" s="28" t="n"/>
+      <c r="G6" s="28" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="19" t="n">
+      <c r="A7" s="29" t="n">
         <v>2</v>
       </c>
-      <c r="B7" s="12" t="inlineStr">
+      <c r="B7" s="30" t="inlineStr">
         <is>
           <t>Cubrir y refrigerar toppings</t>
         </is>
       </c>
-      <c r="C7" s="13" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D7" s="13" t="inlineStr">
-        <is>
-          <t>Cocinero</t>
-        </is>
-      </c>
-      <c r="E7" s="13" t="inlineStr">
+      <c r="C7" s="27" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D7" s="27" t="inlineStr">
+        <is>
+          <t>Cocinero</t>
+        </is>
+      </c>
+      <c r="E7" s="27" t="inlineStr">
         <is>
           <t>22:30</t>
         </is>
       </c>
-      <c r="F7" s="14" t="n"/>
-      <c r="G7" s="14" t="n"/>
+      <c r="F7" s="28" t="n"/>
+      <c r="G7" s="28" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="18" t="n">
+      <c r="A8" s="25" t="n">
         <v>3</v>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B8" s="26" t="inlineStr">
         <is>
           <t>Guardar salsas caseras en recipientes herméticos</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D8" s="9" t="inlineStr">
-        <is>
-          <t>Cocinero</t>
-        </is>
-      </c>
-      <c r="E8" s="9" t="inlineStr">
+      <c r="C8" s="27" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D8" s="27" t="inlineStr">
+        <is>
+          <t>Cocinero</t>
+        </is>
+      </c>
+      <c r="E8" s="27" t="inlineStr">
         <is>
           <t>22:30</t>
         </is>
       </c>
-      <c r="F8" s="10" t="n"/>
-      <c r="G8" s="10" t="n"/>
+      <c r="F8" s="28" t="n"/>
+      <c r="G8" s="28" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="19" t="n">
+      <c r="A9" s="29" t="n">
         <v>4</v>
       </c>
-      <c r="B9" s="12" t="inlineStr">
+      <c r="B9" s="30" t="inlineStr">
         <is>
           <t>Guardar pan sobrante en bolsa hermética</t>
         </is>
       </c>
-      <c r="C9" s="13" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D9" s="13" t="inlineStr">
-        <is>
-          <t>Cocinero</t>
-        </is>
-      </c>
-      <c r="E9" s="13" t="inlineStr">
+      <c r="C9" s="27" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D9" s="27" t="inlineStr">
+        <is>
+          <t>Cocinero</t>
+        </is>
+      </c>
+      <c r="E9" s="27" t="inlineStr">
         <is>
           <t>22:30</t>
         </is>
       </c>
-      <c r="F9" s="14" t="n"/>
-      <c r="G9" s="14" t="n"/>
+      <c r="F9" s="28" t="n"/>
+      <c r="G9" s="28" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="18" t="n">
+      <c r="A10" s="25" t="n">
         <v>5</v>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B10" s="26" t="inlineStr">
         <is>
           <t>Etiquetar todo con fecha</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D10" s="9" t="inlineStr">
-        <is>
-          <t>Cocinero</t>
-        </is>
-      </c>
-      <c r="E10" s="9" t="inlineStr">
+      <c r="C10" s="27" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D10" s="27" t="inlineStr">
+        <is>
+          <t>Cocinero</t>
+        </is>
+      </c>
+      <c r="E10" s="27" t="inlineStr">
         <is>
           <t>22:30</t>
         </is>
       </c>
-      <c r="F10" s="10" t="n"/>
-      <c r="G10" s="10" t="n"/>
+      <c r="F10" s="28" t="n"/>
+      <c r="G10" s="28" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="A11" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">  PLANCHA Y EQUIPOS</t>
         </is>
       </c>
+      <c r="B11" s="24" t="n"/>
+      <c r="C11" s="24" t="n"/>
+      <c r="D11" s="24" t="n"/>
+      <c r="E11" s="24" t="n"/>
+      <c r="F11" s="24" t="n"/>
+      <c r="G11" s="24" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="18" t="n">
+      <c r="A12" s="25" t="n">
         <v>6</v>
       </c>
-      <c r="B12" s="8" t="inlineStr">
+      <c r="B12" s="26" t="inlineStr">
         <is>
           <t>Limpiar plancha/grill a fondo (rasqueta + desengrasante)</t>
         </is>
       </c>
-      <c r="C12" s="9" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D12" s="9" t="inlineStr">
-        <is>
-          <t>Cocinero</t>
-        </is>
-      </c>
-      <c r="E12" s="9" t="inlineStr">
+      <c r="C12" s="27" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D12" s="27" t="inlineStr">
+        <is>
+          <t>Cocinero</t>
+        </is>
+      </c>
+      <c r="E12" s="27" t="inlineStr">
         <is>
           <t>22:30</t>
         </is>
       </c>
-      <c r="F12" s="10" t="n"/>
-      <c r="G12" s="10" t="n"/>
+      <c r="F12" s="28" t="n"/>
+      <c r="G12" s="28" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="19" t="n">
+      <c r="A13" s="29" t="n">
         <v>7</v>
       </c>
-      <c r="B13" s="12" t="inlineStr">
-        <is>
-          <t>Filtrar o cambiar aceite de freidora</t>
-        </is>
-      </c>
-      <c r="C13" s="13" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D13" s="13" t="inlineStr">
-        <is>
-          <t>Cocinero</t>
-        </is>
-      </c>
-      <c r="E13" s="13" t="inlineStr">
+      <c r="B13" s="30" t="inlineStr">
+        <is>
+          <t>Apagar la freidora al terminar el servicio y dejar que el aceite se enfríe; la campana sigue en marcha mientras tanto</t>
+        </is>
+      </c>
+      <c r="C13" s="27" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D13" s="27" t="inlineStr">
+        <is>
+          <t>Cocinero</t>
+        </is>
+      </c>
+      <c r="E13" s="27" t="inlineStr">
         <is>
           <t>22:30</t>
         </is>
       </c>
-      <c r="F13" s="14" t="n"/>
-      <c r="G13" s="14" t="n"/>
+      <c r="F13" s="28" t="n"/>
+      <c r="G13" s="28" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="18" t="n">
+      <c r="A14" s="25" t="n">
         <v>8</v>
       </c>
-      <c r="B14" s="8" t="inlineStr">
-        <is>
-          <t>Apagar freidora, plancha, horno, campana</t>
-        </is>
-      </c>
-      <c r="C14" s="9" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D14" s="9" t="inlineStr">
-        <is>
-          <t>Cocinero</t>
-        </is>
-      </c>
-      <c r="E14" s="9" t="inlineStr">
+      <c r="B14" s="26" t="inlineStr">
+        <is>
+          <t>Filtrar o cambiar el aceite SOLO por debajo de 40 °C, nunca en caliente: al filtrarlo hirviendo salpica y es la quemadura más habitual del cierre</t>
+        </is>
+      </c>
+      <c r="C14" s="27" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D14" s="27" t="inlineStr">
+        <is>
+          <t>Cocinero</t>
+        </is>
+      </c>
+      <c r="E14" s="27" t="inlineStr">
         <is>
           <t>22:45</t>
         </is>
       </c>
-      <c r="F14" s="10" t="n"/>
-      <c r="G14" s="10" t="n"/>
+      <c r="F14" s="28" t="n"/>
+      <c r="G14" s="28" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="19" t="n">
+      <c r="A15" s="25" t="n">
         <v>9</v>
       </c>
-      <c r="B15" s="12" t="inlineStr">
-        <is>
-          <t>Verificar cámaras cerradas y a temperatura</t>
-        </is>
-      </c>
-      <c r="C15" s="13" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D15" s="13" t="inlineStr">
-        <is>
-          <t>Cocinero</t>
-        </is>
-      </c>
-      <c r="E15" s="13" t="inlineStr">
+      <c r="B15" s="26" t="inlineStr">
+        <is>
+          <t>Apagar plancha, horno y campana extractora cuando la freidora y la plancha ya estén frías</t>
+        </is>
+      </c>
+      <c r="C15" s="27" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D15" s="27" t="inlineStr">
+        <is>
+          <t>Cocinero</t>
+        </is>
+      </c>
+      <c r="E15" s="27" t="inlineStr">
         <is>
           <t>22:45</t>
         </is>
       </c>
-      <c r="F15" s="14" t="n"/>
-      <c r="G15" s="14" t="n"/>
+      <c r="F15" s="28" t="n"/>
+      <c r="G15" s="28" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="6" t="inlineStr">
+      <c r="A16" s="29" t="n">
+        <v>10</v>
+      </c>
+      <c r="B16" s="30" t="inlineStr">
+        <is>
+          <t>Verificar cámaras cerradas y a temperatura (refrigeración 0-4 °C) — anota la lectura: ____ °C</t>
+        </is>
+      </c>
+      <c r="C16" s="27" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D16" s="27" t="inlineStr">
+        <is>
+          <t>Cocinero</t>
+        </is>
+      </c>
+      <c r="E16" s="27" t="inlineStr">
+        <is>
+          <t>22:45</t>
+        </is>
+      </c>
+      <c r="F16" s="28" t="n"/>
+      <c r="G16" s="28" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">  LIMPIEZA</t>
         </is>
       </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="19" t="n">
-        <v>10</v>
-      </c>
-      <c r="B17" s="12" t="inlineStr">
+      <c r="B17" s="24" t="n"/>
+      <c r="C17" s="24" t="n"/>
+      <c r="D17" s="24" t="n"/>
+      <c r="E17" s="24" t="n"/>
+      <c r="F17" s="24" t="n"/>
+      <c r="G17" s="24" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="29" t="n">
+        <v>11</v>
+      </c>
+      <c r="B18" s="30" t="inlineStr">
         <is>
           <t>Limpiar línea de montaje y bandejas</t>
         </is>
       </c>
-      <c r="C17" s="13" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D17" s="13" t="inlineStr">
+      <c r="C18" s="27" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D18" s="27" t="inlineStr">
         <is>
           <t>Auxiliar</t>
         </is>
       </c>
-      <c r="E17" s="13" t="inlineStr">
+      <c r="E18" s="27" t="inlineStr">
         <is>
           <t>22:30</t>
         </is>
       </c>
-      <c r="F17" s="14" t="n"/>
-      <c r="G17" s="14" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="18" t="n">
-        <v>11</v>
-      </c>
-      <c r="B18" s="8" t="inlineStr">
+      <c r="F18" s="28" t="n"/>
+      <c r="G18" s="28" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="25" t="n">
+        <v>12</v>
+      </c>
+      <c r="B19" s="26" t="inlineStr">
         <is>
           <t>Fregar utensilios: espátulas, prensas, cuchillos</t>
         </is>
       </c>
-      <c r="C18" s="9" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D18" s="9" t="inlineStr">
+      <c r="C19" s="27" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D19" s="27" t="inlineStr">
         <is>
           <t>Auxiliar</t>
         </is>
       </c>
-      <c r="E18" s="9" t="inlineStr">
+      <c r="E19" s="27" t="inlineStr">
         <is>
           <t>22:30</t>
         </is>
       </c>
-      <c r="F18" s="10" t="n"/>
-      <c r="G18" s="10" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="19" t="n">
-        <v>12</v>
-      </c>
-      <c r="B19" s="12" t="inlineStr">
+      <c r="F19" s="28" t="n"/>
+      <c r="G19" s="28" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="29" t="n">
+        <v>13</v>
+      </c>
+      <c r="B20" s="30" t="inlineStr">
         <is>
           <t>Barrer y fregar suelo de cocina</t>
         </is>
       </c>
-      <c r="C19" s="13" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D19" s="13" t="inlineStr">
+      <c r="C20" s="27" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D20" s="27" t="inlineStr">
         <is>
           <t>Auxiliar</t>
         </is>
       </c>
-      <c r="E19" s="13" t="inlineStr">
+      <c r="E20" s="27" t="inlineStr">
         <is>
           <t>22:45</t>
         </is>
       </c>
-      <c r="F19" s="14" t="n"/>
-      <c r="G19" s="14" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="18" t="n">
-        <v>13</v>
-      </c>
-      <c r="B20" s="8" t="inlineStr">
+      <c r="F20" s="28" t="n"/>
+      <c r="G20" s="28" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="25" t="n">
+        <v>14</v>
+      </c>
+      <c r="B21" s="26" t="inlineStr">
         <is>
           <t>Sacar basura y reciclar (cartón, aceite usado)</t>
         </is>
       </c>
-      <c r="C20" s="9" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D20" s="9" t="inlineStr">
+      <c r="C21" s="27" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D21" s="27" t="inlineStr">
         <is>
           <t>Auxiliar</t>
         </is>
       </c>
-      <c r="E20" s="9" t="inlineStr">
+      <c r="E21" s="27" t="inlineStr">
         <is>
           <t>22:45</t>
         </is>
       </c>
-      <c r="F20" s="10" t="n"/>
-      <c r="G20" s="10" t="n"/>
-    </row>
-    <row r="21">
-      <c r="A21" s="6" t="inlineStr">
+      <c r="F21" s="28" t="n"/>
+      <c r="G21" s="28" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">  PREPARACIÓN MAÑANA</t>
         </is>
       </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="18" t="n">
-        <v>14</v>
-      </c>
-      <c r="B22" s="8" t="inlineStr">
+      <c r="B22" s="24" t="n"/>
+      <c r="C22" s="24" t="n"/>
+      <c r="D22" s="24" t="n"/>
+      <c r="E22" s="24" t="n"/>
+      <c r="F22" s="24" t="n"/>
+      <c r="G22" s="24" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="25" t="n">
+        <v>15</v>
+      </c>
+      <c r="B23" s="26" t="inlineStr">
         <is>
           <t>Preparar patties para mañana (si se hacen con antelación)</t>
         </is>
       </c>
-      <c r="C22" s="9" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D22" s="9" t="inlineStr">
-        <is>
-          <t>Cocinero</t>
-        </is>
-      </c>
-      <c r="E22" s="9" t="inlineStr">
+      <c r="C23" s="27" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D23" s="27" t="inlineStr">
+        <is>
+          <t>Cocinero</t>
+        </is>
+      </c>
+      <c r="E23" s="27" t="inlineStr">
         <is>
           <t>22:00</t>
         </is>
       </c>
-      <c r="F22" s="10" t="n"/>
-      <c r="G22" s="10" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="19" t="n">
-        <v>15</v>
-      </c>
-      <c r="B23" s="12" t="inlineStr">
+      <c r="F23" s="28" t="n"/>
+      <c r="G23" s="28" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="29" t="n">
+        <v>16</v>
+      </c>
+      <c r="B24" s="30" t="inlineStr">
         <is>
           <t>Anotar faltantes para pedido</t>
         </is>
       </c>
-      <c r="C23" s="13" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D23" s="13" t="inlineStr">
-        <is>
-          <t>Cocinero</t>
-        </is>
-      </c>
-      <c r="E23" s="13" t="inlineStr">
+      <c r="C24" s="27" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D24" s="27" t="inlineStr">
+        <is>
+          <t>Cocinero</t>
+        </is>
+      </c>
+      <c r="E24" s="27" t="inlineStr">
         <is>
           <t>22:30</t>
         </is>
       </c>
-      <c r="F23" s="14" t="n"/>
-      <c r="G23" s="14" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="18" t="n">
-        <v>16</v>
-      </c>
-      <c r="B24" s="8" t="inlineStr">
+      <c r="F24" s="28" t="n"/>
+      <c r="G24" s="28" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="29" t="n">
+        <v>17</v>
+      </c>
+      <c r="B25" s="30" t="inlineStr">
+        <is>
+          <t>Anotar las mermas del día (producto, cantidad y motivo): patties pasados de punto o caídos, pan seco, toppings retirados y pedidos devueltos — sin este dato el food cost del mes sale mal</t>
+        </is>
+      </c>
+      <c r="C25" s="27" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D25" s="27" t="inlineStr">
+        <is>
+          <t>Cocinero</t>
+        </is>
+      </c>
+      <c r="E25" s="27" t="inlineStr">
+        <is>
+          <t>22:30</t>
+        </is>
+      </c>
+      <c r="F25" s="28" t="n"/>
+      <c r="G25" s="28" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="25" t="n">
+        <v>18</v>
+      </c>
+      <c r="B26" s="26" t="inlineStr">
         <is>
           <t>Descongelar carne para mañana si es necesario</t>
         </is>
       </c>
-      <c r="C24" s="9" t="inlineStr">
-        <is>
-          <t>Cocina</t>
-        </is>
-      </c>
-      <c r="D24" s="9" t="inlineStr">
-        <is>
-          <t>Cocinero</t>
-        </is>
-      </c>
-      <c r="E24" s="9" t="inlineStr">
+      <c r="C26" s="27" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+      <c r="D26" s="27" t="inlineStr">
+        <is>
+          <t>Cocinero</t>
+        </is>
+      </c>
+      <c r="E26" s="27" t="inlineStr">
         <is>
           <t>22:30</t>
         </is>
       </c>
-      <c r="F24" s="10" t="n"/>
-      <c r="G24" s="10" t="n"/>
-    </row>
-    <row r="25"/>
-    <row r="26">
-      <c r="C26" s="15" t="inlineStr">
-        <is>
-          <t>Completadas:</t>
-        </is>
-      </c>
-      <c r="D26" s="16">
-        <f>COUNTIF(F5:F24,"✓")</f>
+      <c r="F26" s="28" t="n"/>
+      <c r="G26" s="28" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="31" t="n"/>
+      <c r="B27" s="32" t="n"/>
+      <c r="C27" s="27" t="n"/>
+      <c r="D27" s="27" t="n"/>
+      <c r="E27" s="27" t="n"/>
+      <c r="F27" s="28" t="n"/>
+      <c r="G27" s="28" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="31" t="n"/>
+      <c r="B28" s="32" t="n"/>
+      <c r="C28" s="27" t="n"/>
+      <c r="D28" s="27" t="n"/>
+      <c r="E28" s="27" t="n"/>
+      <c r="F28" s="28" t="n"/>
+      <c r="G28" s="28" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="31" t="n"/>
+      <c r="B29" s="32" t="n"/>
+      <c r="C29" s="27" t="n"/>
+      <c r="D29" s="27" t="n"/>
+      <c r="E29" s="27" t="n"/>
+      <c r="F29" s="28" t="n"/>
+      <c r="G29" s="28" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="31" t="n"/>
+      <c r="B30" s="32" t="n"/>
+      <c r="C30" s="27" t="n"/>
+      <c r="D30" s="27" t="n"/>
+      <c r="E30" s="27" t="n"/>
+      <c r="F30" s="28" t="n"/>
+      <c r="G30" s="28" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="31" t="n"/>
+      <c r="B31" s="32" t="n"/>
+      <c r="C31" s="27" t="n"/>
+      <c r="D31" s="27" t="n"/>
+      <c r="E31" s="27" t="n"/>
+      <c r="F31" s="28" t="n"/>
+      <c r="G31" s="28" t="n"/>
+    </row>
+    <row r="32"/>
+    <row r="33">
+      <c r="A33" s="15" t="inlineStr">
+        <is>
+          <t>Tareas completadas:</t>
+        </is>
+      </c>
+      <c r="D33" s="16">
+        <f>COUNTIFS(B5:B31,"?*",F5:F31,"✓")</f>
         <v>0.0</v>
       </c>
-      <c r="E26" s="15" t="inlineStr">
+      <c r="E33" s="15" t="inlineStr">
         <is>
           <t>de</t>
         </is>
       </c>
-      <c r="F26">
-        <f>COUNTIF(B5:B24,"?*")</f>
-        <v>16.0</v>
-      </c>
-    </row>
-    <row r="27"/>
-    <row r="28">
-      <c r="A28" s="4" t="inlineStr">
+      <c r="F33">
+        <f>COUNTIF(B5:B31,"?*")-COUNTIF(F5:F31,"N/A")</f>
+        <v>18.0</v>
+      </c>
+    </row>
+    <row r="34"/>
+    <row r="35">
+      <c r="A35" s="4" t="inlineStr">
         <is>
           <t>Firma encargado/a: _________________________    Hora: _________</t>
         </is>
       </c>
     </row>
-    <row r="29"/>
-    <row r="30">
-      <c r="A30" s="17" t="inlineStr">
-        <is>
-          <t>— Kit de Tareas Recurrentes: Hamburguesería · AI Chef Pro · aichef.pro —</t>
+    <row r="36"/>
+    <row r="37">
+      <c r="A37" s="17" t="inlineStr">
+        <is>
+          <t>— Kit de Tareas Recurrentes · Hamburguesería · AI Chef Pro · aichef.pro</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="A28:G28"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="0" formatRows="0" sort="0"/>
+  <mergeCells count="9">
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A16:G16"/>
+    <mergeCell ref="A17:G17"/>
+    <mergeCell ref="A37:G37"/>
+    <mergeCell ref="A35:G35"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A30:G30"/>
-    <mergeCell ref="A21:G21"/>
+    <mergeCell ref="A11:G11"/>
     <mergeCell ref="A5:G5"/>
-    <mergeCell ref="A11:G11"/>
+    <mergeCell ref="A22:G22"/>
+    <mergeCell ref="A33:C33"/>
   </mergeCells>
-  <conditionalFormatting sqref="A5:G24">
+  <conditionalFormatting sqref="A5:G31">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$F5="✓"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F6 F7 F8 F9 F10 F12 F13 F14 F15 F17 F18 F19 F20 F22 F23 F24" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F6 F7 F8 F9 F10 F12 F13 F14 F15 F16 F18 F19 F20 F21 F23 F24 F25 F26 F27 F28 F29 F30 F31" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Marca no válida" error="Usa el desplegable: ✓, — o N/A. N/A = no aplica, sale del total; — = no hecha, cuenta como pendiente." type="list" errorStyle="stop">
       <formula1>"✓,—,N/A"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2553,7 +3208,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -2618,350 +3273,415 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">  SALA</t>
         </is>
       </c>
+      <c r="B5" s="24" t="n"/>
+      <c r="C5" s="24" t="n"/>
+      <c r="D5" s="24" t="n"/>
+      <c r="E5" s="24" t="n"/>
+      <c r="F5" s="24" t="n"/>
+      <c r="G5" s="24" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="18" t="n">
+      <c r="A6" s="25" t="n">
         <v>1</v>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B6" s="26" t="inlineStr">
         <is>
           <t>Desmontar y limpiar mesas</t>
         </is>
       </c>
-      <c r="C6" s="9" t="inlineStr">
+      <c r="C6" s="27" t="inlineStr">
         <is>
           <t>Sala</t>
         </is>
       </c>
-      <c r="D6" s="9" t="inlineStr">
+      <c r="D6" s="27" t="inlineStr">
         <is>
           <t>Camarero/a</t>
         </is>
       </c>
-      <c r="E6" s="9" t="inlineStr">
+      <c r="E6" s="27" t="inlineStr">
         <is>
           <t>22:30</t>
         </is>
       </c>
-      <c r="F6" s="10" t="n"/>
-      <c r="G6" s="10" t="n"/>
+      <c r="F6" s="28" t="n"/>
+      <c r="G6" s="28" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="19" t="n">
+      <c r="A7" s="29" t="n">
         <v>2</v>
       </c>
-      <c r="B7" s="12" t="inlineStr">
+      <c r="B7" s="30" t="inlineStr">
         <is>
           <t>Barrer y fregar suelo</t>
         </is>
       </c>
-      <c r="C7" s="13" t="inlineStr">
+      <c r="C7" s="27" t="inlineStr">
         <is>
           <t>Sala</t>
         </is>
       </c>
-      <c r="D7" s="13" t="inlineStr">
+      <c r="D7" s="27" t="inlineStr">
         <is>
           <t>Auxiliar</t>
         </is>
       </c>
-      <c r="E7" s="13" t="inlineStr">
+      <c r="E7" s="27" t="inlineStr">
         <is>
           <t>22:45</t>
         </is>
       </c>
-      <c r="F7" s="14" t="n"/>
-      <c r="G7" s="14" t="n"/>
+      <c r="F7" s="28" t="n"/>
+      <c r="G7" s="28" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="18" t="n">
+      <c r="A8" s="25" t="n">
         <v>3</v>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B8" s="26" t="inlineStr">
         <is>
           <t>Reponer condimentos para mañana (kétchup, mostaza)</t>
         </is>
       </c>
-      <c r="C8" s="9" t="inlineStr">
+      <c r="C8" s="27" t="inlineStr">
         <is>
           <t>Sala</t>
         </is>
       </c>
-      <c r="D8" s="9" t="inlineStr">
+      <c r="D8" s="27" t="inlineStr">
         <is>
           <t>Camarero/a</t>
         </is>
       </c>
-      <c r="E8" s="9" t="inlineStr">
+      <c r="E8" s="27" t="inlineStr">
         <is>
           <t>22:30</t>
         </is>
       </c>
-      <c r="F8" s="10" t="n"/>
-      <c r="G8" s="10" t="n"/>
+      <c r="F8" s="28" t="n"/>
+      <c r="G8" s="28" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="6" t="inlineStr">
+      <c r="A9" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">  DELIVERY Y CAJA</t>
         </is>
       </c>
+      <c r="B9" s="24" t="n"/>
+      <c r="C9" s="24" t="n"/>
+      <c r="D9" s="24" t="n"/>
+      <c r="E9" s="24" t="n"/>
+      <c r="F9" s="24" t="n"/>
+      <c r="G9" s="24" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="18" t="n">
+      <c r="A10" s="25" t="n">
         <v>4</v>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B10" s="26" t="inlineStr">
         <is>
           <t>Apagar tablets de delivery</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
+      <c r="C10" s="27" t="inlineStr">
         <is>
           <t>Sala</t>
         </is>
       </c>
-      <c r="D10" s="9" t="inlineStr">
+      <c r="D10" s="27" t="inlineStr">
         <is>
           <t>Encargado/a</t>
         </is>
       </c>
-      <c r="E10" s="9" t="inlineStr">
+      <c r="E10" s="27" t="inlineStr">
         <is>
           <t>22:30</t>
         </is>
       </c>
-      <c r="F10" s="10" t="n"/>
-      <c r="G10" s="10" t="n"/>
+      <c r="F10" s="28" t="n"/>
+      <c r="G10" s="28" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="19" t="n">
+      <c r="A11" s="29" t="n">
         <v>5</v>
       </c>
-      <c r="B11" s="12" t="inlineStr">
+      <c r="B11" s="30" t="inlineStr">
         <is>
           <t>Contar packaging restante</t>
         </is>
       </c>
-      <c r="C11" s="13" t="inlineStr">
+      <c r="C11" s="27" t="inlineStr">
         <is>
           <t>Almacén</t>
         </is>
       </c>
-      <c r="D11" s="13" t="inlineStr">
+      <c r="D11" s="27" t="inlineStr">
         <is>
           <t>Encargado/a</t>
         </is>
       </c>
-      <c r="E11" s="13" t="inlineStr">
+      <c r="E11" s="27" t="inlineStr">
         <is>
           <t>22:30</t>
         </is>
       </c>
-      <c r="F11" s="14" t="n"/>
-      <c r="G11" s="14" t="n"/>
+      <c r="F11" s="28" t="n"/>
+      <c r="G11" s="28" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="18" t="n">
+      <c r="A12" s="25" t="n">
         <v>6</v>
       </c>
-      <c r="B12" s="8" t="inlineStr">
+      <c r="B12" s="26" t="inlineStr">
         <is>
           <t>Cuadrar caja (efectivo + tarjeta + delivery)</t>
         </is>
       </c>
-      <c r="C12" s="9" t="inlineStr">
+      <c r="C12" s="27" t="inlineStr">
         <is>
           <t>Office</t>
         </is>
       </c>
-      <c r="D12" s="9" t="inlineStr">
+      <c r="D12" s="27" t="inlineStr">
         <is>
           <t>Encargado/a</t>
         </is>
       </c>
-      <c r="E12" s="9" t="inlineStr">
+      <c r="E12" s="27" t="inlineStr">
         <is>
           <t>22:45</t>
         </is>
       </c>
-      <c r="F12" s="10" t="n"/>
-      <c r="G12" s="10" t="n"/>
+      <c r="F12" s="28" t="n"/>
+      <c r="G12" s="28" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="19" t="n">
+      <c r="A13" s="29" t="n">
         <v>7</v>
       </c>
-      <c r="B13" s="12" t="inlineStr">
+      <c r="B13" s="30" t="inlineStr">
         <is>
           <t>Anotar incidencias</t>
         </is>
       </c>
-      <c r="C13" s="13" t="inlineStr">
+      <c r="C13" s="27" t="inlineStr">
         <is>
           <t>Office</t>
         </is>
       </c>
-      <c r="D13" s="13" t="inlineStr">
+      <c r="D13" s="27" t="inlineStr">
         <is>
           <t>Encargado/a</t>
         </is>
       </c>
-      <c r="E13" s="13" t="inlineStr">
+      <c r="E13" s="27" t="inlineStr">
         <is>
           <t>22:45</t>
         </is>
       </c>
-      <c r="F13" s="14" t="n"/>
-      <c r="G13" s="14" t="n"/>
+      <c r="F13" s="28" t="n"/>
+      <c r="G13" s="28" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="inlineStr">
+      <c r="A14" s="23" t="inlineStr">
         <is>
           <t xml:space="preserve">  CIERRE FINAL</t>
         </is>
       </c>
+      <c r="B14" s="24" t="n"/>
+      <c r="C14" s="24" t="n"/>
+      <c r="D14" s="24" t="n"/>
+      <c r="E14" s="24" t="n"/>
+      <c r="F14" s="24" t="n"/>
+      <c r="G14" s="24" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="19" t="n">
+      <c r="A15" s="29" t="n">
         <v>8</v>
       </c>
-      <c r="B15" s="12" t="inlineStr">
+      <c r="B15" s="30" t="inlineStr">
         <is>
           <t>Limpieza final de baños</t>
         </is>
       </c>
-      <c r="C15" s="13" t="inlineStr">
+      <c r="C15" s="27" t="inlineStr">
         <is>
           <t>Baños</t>
         </is>
       </c>
-      <c r="D15" s="13" t="inlineStr">
+      <c r="D15" s="27" t="inlineStr">
         <is>
           <t>Auxiliar</t>
         </is>
       </c>
-      <c r="E15" s="13" t="inlineStr">
+      <c r="E15" s="27" t="inlineStr">
         <is>
           <t>22:45</t>
         </is>
       </c>
-      <c r="F15" s="14" t="n"/>
-      <c r="G15" s="14" t="n"/>
+      <c r="F15" s="28" t="n"/>
+      <c r="G15" s="28" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="18" t="n">
+      <c r="A16" s="25" t="n">
         <v>9</v>
       </c>
-      <c r="B16" s="8" t="inlineStr">
+      <c r="B16" s="26" t="inlineStr">
         <is>
           <t>Apagar luces, climatización, música</t>
         </is>
       </c>
-      <c r="C16" s="9" t="inlineStr">
+      <c r="C16" s="27" t="inlineStr">
         <is>
           <t>Sala</t>
         </is>
       </c>
-      <c r="D16" s="9" t="inlineStr">
+      <c r="D16" s="27" t="inlineStr">
         <is>
           <t>Encargado/a</t>
         </is>
       </c>
-      <c r="E16" s="9" t="inlineStr">
+      <c r="E16" s="27" t="inlineStr">
         <is>
           <t>23:00</t>
         </is>
       </c>
-      <c r="F16" s="10" t="n"/>
-      <c r="G16" s="10" t="n"/>
+      <c r="F16" s="28" t="n"/>
+      <c r="G16" s="28" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="19" t="n">
+      <c r="A17" s="29" t="n">
         <v>10</v>
       </c>
-      <c r="B17" s="12" t="inlineStr">
+      <c r="B17" s="30" t="inlineStr">
         <is>
           <t>Activar alarma y cerrar</t>
         </is>
       </c>
-      <c r="C17" s="13" t="inlineStr">
+      <c r="C17" s="27" t="inlineStr">
         <is>
           <t>Sala</t>
         </is>
       </c>
-      <c r="D17" s="13" t="inlineStr">
+      <c r="D17" s="27" t="inlineStr">
         <is>
           <t>Encargado/a</t>
         </is>
       </c>
-      <c r="E17" s="13" t="inlineStr">
+      <c r="E17" s="27" t="inlineStr">
         <is>
           <t>23:00</t>
         </is>
       </c>
-      <c r="F17" s="14" t="n"/>
-      <c r="G17" s="14" t="n"/>
-    </row>
-    <row r="18"/>
+      <c r="F17" s="28" t="n"/>
+      <c r="G17" s="28" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="31" t="n"/>
+      <c r="B18" s="32" t="n"/>
+      <c r="C18" s="27" t="n"/>
+      <c r="D18" s="27" t="n"/>
+      <c r="E18" s="27" t="n"/>
+      <c r="F18" s="28" t="n"/>
+      <c r="G18" s="28" t="n"/>
+    </row>
     <row r="19">
-      <c r="C19" s="15" t="inlineStr">
-        <is>
-          <t>Completadas:</t>
-        </is>
-      </c>
-      <c r="D19" s="16">
-        <f>COUNTIF(F5:F17,"✓")</f>
+      <c r="A19" s="31" t="n"/>
+      <c r="B19" s="32" t="n"/>
+      <c r="C19" s="27" t="n"/>
+      <c r="D19" s="27" t="n"/>
+      <c r="E19" s="27" t="n"/>
+      <c r="F19" s="28" t="n"/>
+      <c r="G19" s="28" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="31" t="n"/>
+      <c r="B20" s="32" t="n"/>
+      <c r="C20" s="27" t="n"/>
+      <c r="D20" s="27" t="n"/>
+      <c r="E20" s="27" t="n"/>
+      <c r="F20" s="28" t="n"/>
+      <c r="G20" s="28" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="31" t="n"/>
+      <c r="B21" s="32" t="n"/>
+      <c r="C21" s="27" t="n"/>
+      <c r="D21" s="27" t="n"/>
+      <c r="E21" s="27" t="n"/>
+      <c r="F21" s="28" t="n"/>
+      <c r="G21" s="28" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="31" t="n"/>
+      <c r="B22" s="32" t="n"/>
+      <c r="C22" s="27" t="n"/>
+      <c r="D22" s="27" t="n"/>
+      <c r="E22" s="27" t="n"/>
+      <c r="F22" s="28" t="n"/>
+      <c r="G22" s="28" t="n"/>
+    </row>
+    <row r="23"/>
+    <row r="24">
+      <c r="A24" s="15" t="inlineStr">
+        <is>
+          <t>Tareas completadas:</t>
+        </is>
+      </c>
+      <c r="D24" s="16">
+        <f>COUNTIFS(B5:B22,"?*",F5:F22,"✓")</f>
         <v>0.0</v>
       </c>
-      <c r="E19" s="15" t="inlineStr">
+      <c r="E24" s="15" t="inlineStr">
         <is>
           <t>de</t>
         </is>
       </c>
-      <c r="F19">
-        <f>COUNTIF(B5:B17,"?*")</f>
+      <c r="F24">
+        <f>COUNTIF(B5:B22,"?*")-COUNTIF(F5:F22,"N/A")</f>
         <v>10.0</v>
       </c>
     </row>
-    <row r="20"/>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
+    <row r="25"/>
+    <row r="26">
+      <c r="A26" s="4" t="inlineStr">
         <is>
           <t>Firma encargado/a: _________________________    Hora: _________</t>
         </is>
       </c>
     </row>
-    <row r="22"/>
-    <row r="23">
-      <c r="A23" s="17" t="inlineStr">
-        <is>
-          <t>— Kit de Tareas Recurrentes: Hamburguesería · AI Chef Pro · aichef.pro —</t>
+    <row r="27"/>
+    <row r="28">
+      <c r="A28" s="17" t="inlineStr">
+        <is>
+          <t>— Kit de Tareas Recurrentes · Hamburguesería · AI Chef Pro · aichef.pro</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="0" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="0" formatCells="0" formatRows="0" sort="0"/>
+  <mergeCells count="8">
+    <mergeCell ref="A28:G28"/>
     <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A14:G14"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A14:G14"/>
-    <mergeCell ref="A21:G21"/>
     <mergeCell ref="A9:G9"/>
-    <mergeCell ref="A23:G23"/>
+    <mergeCell ref="A24:C24"/>
     <mergeCell ref="A5:G5"/>
+    <mergeCell ref="A26:G26"/>
   </mergeCells>
-  <conditionalFormatting sqref="A5:G17">
+  <conditionalFormatting sqref="A5:G22">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$F5="✓"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation sqref="F6 F7 F8 F10 F11 F12 F13 F15 F16 F17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F6 F7 F8 F10 F11 F12 F13 F15 F16 F17 F18 F19 F20 F21 F22" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Marca no válida" error="Usa el desplegable: ✓, — o N/A. N/A = no aplica, sale del total; — = no hecha, cuenta como pendiente." type="list" errorStyle="stop">
       <formula1>"✓,—,N/A"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>